<commit_message>
clean dead and unnecessary code, reduce hardcoded values, add prompt for LLM, scrape 100 reports for RAG
</commit_message>
<xml_diff>
--- a/data/raw/Non Chinese data from refinery to Companies (Apple, etc...).xlsx
+++ b/data/raw/Non Chinese data from refinery to Companies (Apple, etc...).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momo/HackSummit/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0535227E-89CE-3248-8F35-0D199CEB8843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DF7612-D992-764A-B50D-3BD967837F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -493,7 +493,7 @@
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="80.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="85.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.33203125" bestFit="1" customWidth="1"/>

</xml_diff>